<commit_message>
Status sheet: the designer's revised debuff rules
Stack debuffs now read as "a stack is 5 tempo" (one stack dissipates
every 5 tempo on the debuff's own clock; hits, moves and card plays no
longer consume them); Disarm, Rooted, Silence and the enemy Disarm,
Root and Curse are additive timers; enemy Wear Down lasts 2 enemy
attacks; enemy Shock arcs to a neighbour; enemy Cold thaws 3 per cycle;
Lowered Physical Defense is grouped stacks; Locked holds several cards.
The code change to match follows.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013Z9NtQ2TzQNePbijiyLyp4
</commit_message>
<xml_diff>
--- a/docs/STATUS_EFFECTS.xlsx
+++ b/docs/STATUS_EFFECTS.xlsx
@@ -3454,7 +3454,7 @@
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Giant Beaver 'Chomp' (3t); Cerberus 'Venom Tail' (15t, also knocks 3 cards from hand); Inflamed Minotaur 'Bull Rush' (5t, chance = spaces x4%); self: Stone Encase [Strap of Stone] (5t), Cryonics (15t on the iced ally or self)</t>
+          <t>Giant Beaver 'Chomp' (3t); Cerberus 'Venom Tail' (15t, also knocks 3 cards from hand); Inflamed Minotaur 'Bull Rush' (5t, chance = spaces x4%); Weregoat Charge landing (3t); self: Stone Encase [Strap of Stone] (5t), Cryonics (15t on the iced ally or self)</t>
         </is>
       </c>
       <c r="J3" s="39" t="inlineStr">
@@ -3486,12 +3486,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Cannot play attack cards.</t>
+          <t>Cannot play attack cards or use the auto-attack button.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Timed (tempo)</t>
+          <t>Timed (tempo), additive</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -3501,7 +3501,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Not stackable: re-applying keeps the longer timer</t>
+          <t>Stackable: re-applying ADDS the new duration</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -3544,17 +3544,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Timed (tempo)</t>
+          <t>Timed (tempo), additive</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>15 tempo</t>
+          <t>5 tempo</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Not stackable: re-applying keeps the longer timer</t>
+          <t>Stackable: re-applying ADDS the new duration</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -3662,7 +3662,7 @@
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>White Manticore 'Stinger' (8)</t>
+          <t>White Manticore 'Stinger' (8); Sewer Cobra Venom Spray (8, cone) and its poison-back (3)</t>
         </is>
       </c>
       <c r="J7" s="43" t="inlineStr">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>15 tempo (sources use 10)</t>
+          <t>10 tempo</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -3809,7 +3809,7 @@
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Cerberus Venom Tail aftermath when the stun ends (10t); self: Succumb (10t)</t>
+          <t>Cerberus Venom Tail aftermath when the stun ends (10t); self: Succumb (10t); Demon Cuff (15t); Mind Eater Manipulate Mind Space (15t)</t>
         </is>
       </c>
       <c r="J10" s="46" t="inlineStr">
@@ -3886,12 +3886,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Movement costs 3 tempo per tile instead of 1; each tile moved burns a stack. The clock-timed variant lasts N tempo and burns no stacks.</t>
+          <t>Movement costs 3 tempo per tile instead of 1 while any stack remains. Each stack lasts 5 tempo; tiles moved do not consume stacks. The clock-timed variant (Approach, Snow Wraith, Fire Web) lasts N tempo instead.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Stacks (never expires by the clock) or Timed (tempo)</t>
+          <t>Stacks, 5 tempo each (own clock), or Timed (tempo)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -3907,7 +3907,7 @@
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Ice Mage 'Frost Bolt' (1); Spiked Web trap in cave interiors (2, plus 5 damage); self: Petey the Pet Rock while in hand (held at 2), Approach (timed, 10t)</t>
+          <t>Ice Mage 'Frost Bolt' (1); Spiked Web trap in cave interiors (2, plus 5 damage); Snow Wraith (timed 3t); Magma Spider Fire Web (while inside); self: Petey the Pet Rock while in hand (held at 2), Approach (timed, 10t)</t>
         </is>
       </c>
       <c r="J12" s="48" t="inlineStr">
@@ -3935,12 +3935,12 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Attack cards cost 15 more mana; each attack card played burns a stack. The clock-timed variant lasts N tempo instead.</t>
+          <t>Attack cards cost 15 more mana while any stack remains; each stack lasts 5 tempo (attack cards do not consume stacks). The clock-timed variant (Tower Shield) lasts N tempo instead.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Stacks (never expires by the clock) or Timed (tempo)</t>
+          <t>Stacks, 5 tempo each (own clock), or Timed (tempo)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -4005,7 +4005,7 @@
       <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Self only: Succumb (1, 10t)</t>
+          <t>Self only: Succumb (1, 10t); Release Soul held in hand (held at 1 stack)</t>
         </is>
       </c>
       <c r="J14" s="50" t="inlineStr">
@@ -4054,7 +4054,7 @@
       <c r="H15" s="2" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>None in the live game</t>
+          <t>Infected Hunter Net Throw (1 stack per card in hand)</t>
         </is>
       </c>
       <c r="J15" s="51" t="inlineStr">
@@ -4092,7 +4092,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>15 tempo (source uses 25)</t>
+          <t>25 tempo (Mind Eater: until played)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -4103,7 +4103,7 @@
       <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Necromancer 'Dark Bolt' (2 hexes, +30 mana each, 25t)</t>
+          <t>Necromancer 'Dark Bolt' (2 hexes, +30 mana each, 25t); Mind Eater Mind Slow (+20 on every card in hand, until played)</t>
         </is>
       </c>
       <c r="J16" s="52" t="inlineStr">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>One random card in hand cannot be played.</t>
+          <t>One random card in hand cannot be played. Each Locked is its own instance on its own card, so several cards can be locked at once.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Not stackable: re-applying keeps the longer timer</t>
+          <t>Never merges: each application locks another card</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -4185,17 +4185,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Timed (tempo)</t>
+          <t>Timed (tempo), additive</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>15 tempo (source uses 8)</t>
+          <t>5 tempo (Treant applies 8)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Not stackable: re-applying keeps the longer timer</t>
+          <t>Stackable: re-applying ADDS the new duration</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4229,12 +4229,12 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>30% chance to discard a random card whenever you play a card; each card played burns a stack.</t>
+          <t>30% chance to discard a random card whenever you play a card, while any stack remains; each stack lasts 5 tempo (card plays do not consume stacks).</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Stacks (never expires by the clock)</t>
+          <t>Stacks, 5 tempo each (own clock)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -4250,7 +4250,7 @@
       <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>White Manticore 'Stinger' (3 stacks)</t>
+          <t>White Manticore 'Stinger' (3 stacks = 15 tempo)</t>
         </is>
       </c>
       <c r="J19" s="55" t="inlineStr">
@@ -4278,28 +4278,28 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Take 30% more damage from the next X attacks (not from damage-over-time ticks); one stack per hit.</t>
+          <t>Take 30% more damage while any stack remains. Each stack lasts 5 tempo: 1 stack dissipates every 5 tempo on the debuff's own clock. Hits do not consume stacks.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Stacks (value) and also expires when its timer ends</t>
+          <t>Stacks, 5 tempo each (own clock)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>15 tempo</t>
+          <t>stacks = value applied</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Stackable: re-applying adds the value and keeps the longer timer</t>
+          <t>Stackable: re-applying adds stacks</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Giant Beaver 'Tail Whip' (5, 15t); Large Bear 'Roar' (1 to every player unit within 4); Cerberus venom aftermath (2); Inflamed Minotaur Bull Rush (1 to the victim and to everything trampled); self: Bloodlust (3, until cleansed)</t>
+          <t>Giant Beaver 'Tail Whip' (5); Large Bear 'Roar' (1 to every player unit within 4); Cerberus venom aftermath (2); Inflamed Minotaur Bull Rush (1 to the victim and to everything trampled); self: Bloodlust (3)</t>
         </is>
       </c>
       <c r="J20" s="56" t="inlineStr">
@@ -4327,28 +4327,28 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Armor decays an extra 2 per cycle; lose 1 stack at the end of each cycle.</t>
+          <t>Armor decays an extra 2 per cycle while any stack remains. Each stack lasts 5 tempo: 1 stack dissipates every 5 tempo on the debuff's own clock.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Value decays 1 per cycle; also expires when its timer ends</t>
+          <t>Stacks, 5 tempo each (own clock)</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>15 tempo</t>
+          <t>1 stack = 5 tempo</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Stackable: re-applying adds the value and keeps the longer timer</t>
+          <t>Stackable: re-applying adds stacks</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Ice Troll, every hit incl. 'Club' and 'Clobber' (1, 15t)</t>
+          <t>Ice Troll, every hit incl. 'Club' and 'Clobber' (1)</t>
         </is>
       </c>
       <c r="J21" s="57" t="inlineStr">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>15 tempo</t>
+          <t>5 tempo</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -4397,7 +4397,7 @@
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Ice Troll, every hit (1, 15t); if a hit freezes you, 'Clobber' (50 damage) follows</t>
+          <t>Ice Troll, every hit (1, 5t); if a hit freezes you, 'Clobber' (50 damage) follows; Snow Wraith Snowball (2, 5t)</t>
         </is>
       </c>
       <c r="J22" s="58" t="inlineStr">
@@ -4425,28 +4425,28 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>X% chance for your attacks to miss.</t>
+          <t>80% chance for your attacks to miss (BLIND_MISS). Each stack lasts 5 tempo.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Timed (tempo)</t>
+          <t>Stacks, 5 tempo each (own clock)</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>BLIND_MISS = 80%, 15 tempo (source uses 5)</t>
+          <t>1 stack = 5 tempo</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Not stackable: re-applying keeps the longer timer</t>
+          <t>Stackable: re-applying adds stacks</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Giant Hawk 'Swoop' (20% chance, 5t)</t>
+          <t>Giant Hawk 'Swoop' (20% chance, 1 stack)</t>
         </is>
       </c>
       <c r="J23" s="59" t="inlineStr">
@@ -4478,12 +4478,12 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Deal 30% less damage; each attack burns a stack. Mirrors the enemy-side Weaken.</t>
+          <t>Deal 30% less damage while any stack remains; each stack lasts 5 tempo. Attacks do not consume stacks.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Stacks (never expires by the clock)</t>
+          <t>Stacks, 5 tempo each (own clock)</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -4499,7 +4499,7 @@
       <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Inflamed Minotaur Bull Rush, on the same roll as its stun (1 stack)</t>
+          <t>Inflamed Minotaur Bull Rush, on the same roll as its stun (1 stack); Roc Eye Scrape (2 stacks)</t>
         </is>
       </c>
       <c r="J24" s="15" t="inlineStr">
@@ -4637,9 +4637,10 @@
           <t>Timed (tempo)</t>
         </is>
       </c>
-      <c r="F27" s="2">
-        <f> the tempo spent on the swap</f>
-        <v/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>the tempo spent on the gear swap</t>
+        </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
@@ -4926,12 +4927,12 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Each movement action costs +2 tempo (SLOWED_TEMPO_PER_TILE - 1) and burns one stack, regardless of tiles covered. Each stack also shortens the Inflamed Minotaur's Labyrinth Leap by 1.</t>
+          <t>Each movement action costs +2 tempo while any stack remains; each stack lasts 5 tempo on its own clock (moves do not consume stacks). Each stack also shortens the Inflamed Minotaur's Labyrinth Leap by 1.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Stacks (never expires by the clock)</t>
+          <t>Stacks, 5 tempo each (own clock)</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -4983,12 +4984,12 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Cannot attack for N tempo.</t>
+          <t>Cannot attack.</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Timed (tempo)</t>
+          <t>Timed (tempo), additive</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -4998,7 +4999,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Re-applying OVERWRITES the timer (does not keep the longer one)</t>
+          <t>Stackable: re-applying ADDS the new duration</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -5040,17 +5041,17 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Skips its next N attack actions.</t>
+          <t>Each stack adds 5 tempo of Disarm (the enemy cannot attack).</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Charges (one per skipped attack)</t>
+          <t>Timed (tempo), 5 tempo per stack</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>1 attack</t>
+          <t>1 stack = 5 tempo</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -5293,12 +5294,12 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Stacking; at 5 it becomes Frozen for 5 tempo and Cold resets. Thaws 1 stack per cycle. Under Element Pollination each tick also deals doubling damage.</t>
+          <t>Stacking; at 5 it becomes Frozen for 5 tempo and Cold resets. Thaws 3 stacks per cycle. Under Element Pollination each tick also deals doubling damage.</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Stacks (thaw 1 per cycle)</t>
+          <t>Stacks (thaw 3 per cycle)</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -5452,7 +5453,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Takes damage equal to its stacks each cycle, then loses 1 stack. Under Element Pollination 5 stacks become a 5-tempo stun.</t>
+          <t>Takes damage equal to its stacks each cycle, deals damage equal to stack to a nearby enemy (2 squares away), then loses 1 stack. Under Element Pollination 5 stacks become a 5-tempo stun.</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -5562,12 +5563,12 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Your next hits deal +30%; one stack burns per hit.</t>
+          <t>Your hits deal +30% while any stack remains; each stack lasts 5 tempo on its own clock (hits do not consume stacks).</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Stacks (one per hit)</t>
+          <t>Stacks, 5 tempo each (own clock)</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -5615,12 +5616,12 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Deals 30% less damage; one stack burns per attack. Zone variant (Territorial Mark): no stacks, lasts while it stands in the smoke.</t>
+          <t>Deals 30% less damage while any stack remains; each stack lasts 5 tempo on its own clock (attacks do not consume stacks). Zone variant (Territorial Mark): no stacks, lasts while it stands in the smoke.</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Stacks (one per attack) or zone</t>
+          <t>Stacks, 5 tempo each (own clock), or zone</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -5726,17 +5727,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Timed (tempo)</t>
+          <t>Timed (tempo), additive</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>5-25 tempo by source</t>
+          <t>5 tempo per stack</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Keeps the longer timer</t>
+          <t>Stackable: re-applying ADDS the new duration</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -5779,17 +5780,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Timed (tempo)</t>
+          <t>Timed (tempo), additive</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>5 tempo</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Keeps the longer timer</t>
+          <t>Stackable: re-applying ADDS the new duration</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -6179,12 +6180,12 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Timed (tempo)</t>
+          <t>2 enemy attacks</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>15 tempo</t>
+          <t>2 enemy attacks</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -6223,22 +6224,22 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Physical hits land X% harder on it for N tempo.</t>
+          <t>Physical hits land X% harder on it. Applied as groups of stacks; each stack lasts 5 tempo on its group's own clock.</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Timed (tempo)</t>
+          <t>Stacks, 5 tempo each (own clock)</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>1-15%, 5 tempo</t>
+          <t>1-15%, 1 stack (Mad Scientist)</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>A stronger % replaces a weaker one; the timer refreshes</t>
+          <t>A stronger % overrides a weaker % while both groups have stacks. For instance, 4 stacks at 10% plus an ally's 2 stacks at 50%: the 50% applies until its 2 stacks are out, then the remaining 10% stacks apply.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Status sheet: the designer's rulings on the audit bugs
Mark keeps the longer timer; Stun blocks every action but Wait; Blind
also misses the basic attack and Flash Cut; Weighted taxes card plays
only; hexes and locks belong to their card; Exposed clears on armor
gain; Tripped wears off; Enlightened and Resilient are separate
instances; Haste spends a charge on every move. Code follows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013Z9NtQ2TzQNePbijiyLyp4
</commit_message>
<xml_diff>
--- a/docs/STATUS_EFFECTS.xlsx
+++ b/docs/STATUS_EFFECTS.xlsx
@@ -1368,7 +1368,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Not stackable: re-applying keeps the higher charge count (never adds); a higher % replaces a lower one</t>
+          <t>Separate instances: each application keeps its own % and charges; the highest % applies and spends its own charges first, then the next</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>+X tempo-free tiles on each of your next Y (non-Flash) moves; one charge per move action.</t>
+          <t>+X tempo-free tiles on each of your next Y moves; every move spends a charge, Flash moves included.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Not stackable: keeps the longer timer; a stronger % replaces a weaker one</t>
+          <t>Separate instances per damage type: a hit uses the best instance that covers its type (an untyped one covers all); the same type keeps the stronger % and the longer timer</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Cannot take any actions: no cards, no movement.</t>
+          <t>Cannot take any actions: no cards, movement, basic attack or block, Sidestep, Flash Cut, gauntlet skills, Brain draws or peeks, or gear swaps. Only the Wait button works; reactions that fire automatically still fire.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Cards cost 2 more tempo; each card played burns a stack.</t>
+          <t>Card plays cost 2 more tempo (hand, Quiver and Manifest plays); each card played burns a stack. The basic attack and basic block are not cards and are not taxed.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>One random card in your hand costs +X mana until it is played; playing it clears every hex on it. Each hex is its own instance on its own card.</t>
+          <t>One card in your hand costs +X mana until it is played. A hex belongs to its card: it leaves with the card if the card leaves the hand any other way. Each hex is its own instance on its own card.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>One random card in hand cannot be played. Each Locked is its own instance on its own card, so several cards can be locked at once.</t>
+          <t>One card in hand cannot be played. A lock belongs to its card and leaves with it. Each Locked is its own instance on its own card, so several cards can be locked at once.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -4425,7 +4425,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>80% chance for your attacks to miss (BLIND_MISS). Each stack lasts 5 tempo.</t>
+          <t>80% chance for your attacks to miss (BLIND_MISS): attack cards, the basic attack and Flash Cut. Each stack lasts 5 tempo.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -5105,7 +5105,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Re-applying OVERWRITES the timer</t>
+          <t>Not stackable: re-applying keeps the longer timer (the +1 riders never shorten it)</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -5674,7 +5674,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Timed (tempo)</t>
+          <t>Timed (tempo); wears off on its own</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -6127,7 +6127,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Flag until it gains armor again</t>
+          <t>Flag until it gains armor again (cleared on any armor gain)</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Status sheet: Exposed cooldown and card-bound countdowns
Exposed has a 10-tempo cooldown per unit; hexes and locks stay on their
card, keep counting in the discard and draw piles, and freeze in jail.
Code follows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013Z9NtQ2TzQNePbijiyLyp4
</commit_message>
<xml_diff>
--- a/docs/STATUS_EFFECTS.xlsx
+++ b/docs/STATUS_EFFECTS.xlsx
@@ -4082,7 +4082,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>One card in your hand costs +X mana until it is played. A hex belongs to its card: it leaves with the card if the card leaves the hand any other way. Each hex is its own instance on its own card.</t>
+          <t>One card in your hand costs +X mana until it is played. A hex stays on its card wherever the card goes: its timer keeps running in the discard and draw piles and freezes while the card is jailed, and it is still there if the card comes back. Each hex is its own instance on its own card.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>One card in hand cannot be played. A lock belongs to its card and leaves with it. Each Locked is its own instance on its own card, so several cards can be locked at once.</t>
+          <t>One card in hand cannot be played. A lock stays on its card wherever the card goes: its timer keeps running in the discard and draw piles and freezes while the card is jailed. Each Locked is its own instance on its own card, so several cards can be locked at once.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Its armor was broken through to 0. Fires on-expose passives (Easy Target, Premeditated) and reactions.</t>
+          <t>Its armor was broken through to 0. Fires on-expose passives (Easy Target, Premeditated) and reactions. Each unit then has a 10-tempo cooldown: another break within 10 tempo is not an Exposed and fires nothing.</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -6137,7 +6137,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>n/a (10-tempo cooldown per unit before it can trigger again)</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>

</xml_diff>